<commit_message>
refactor(io): Add a partial reader for CT_Rst for SST
Current SST is read through OpenXML SDK API. That requires a lot of allocations, because it builds an intermediate representation that is used to convert into the final ClosedXML internal representation.

This creates a forward-onyl reader that can read CT_Rst elements that are used in several places of the XML (SST, cell inlined text or comments).

The reader provides a single method to parse the CT_Rst and that creates either text or immutable rich text.

The SST is read into a temporary table that is used during sheet data loading, because just creating SST directly would cause a lot of changes in the test files. That is left for the later.

The test file UsingRichText has one switched string item index, no semantic change.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Styles/UsingRichText.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Styles/UsingRichText.xlsx
@@ -48,63 +48,63 @@
     </x:r>
   </x:si>
   <x:si>
-    <x:t>" BIG " is Bold.</x:t>
+    <x:r>
+      <x:rPr>
+        <x:vertAlign val="baseline"/>
+        <x:sz val="11"/>
+        <x:color rgb="FFFF0000"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+      </x:rPr>
+      <x:t>Hell</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:u val="single"/>
+        <x:vertAlign val="baseline"/>
+        <x:sz val="11"/>
+        <x:color rgb="FFFF0000"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+      </x:rPr>
+      <x:t>o</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:b/>
+        <x:u val="single"/>
+        <x:vertAlign val="baseline"/>
+        <x:sz val="11"/>
+        <x:color rgb="FF0000FF"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+      </x:rPr>
+      <x:t xml:space="preserve"> BIG </x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:u val="single"/>
+        <x:vertAlign val="baseline"/>
+        <x:sz val="11"/>
+        <x:color rgb="FFFF0000"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+      </x:rPr>
+      <x:t>W</x:t>
+    </x:r>
+    <x:r>
+      <x:rPr>
+        <x:vertAlign val="baseline"/>
+        <x:sz val="11"/>
+        <x:color rgb="FFFF0000"/>
+        <x:rFont val="Calibri"/>
+        <x:family val="2"/>
+      </x:rPr>
+      <x:t>orld</x:t>
+    </x:r>
   </x:si>
   <x:si>
-    <x:r>
-      <x:rPr>
-        <x:vertAlign val="baseline"/>
-        <x:sz val="11"/>
-        <x:color rgb="FFFF0000"/>
-        <x:rFont val="Calibri"/>
-        <x:family val="2"/>
-      </x:rPr>
-      <x:t>Hell</x:t>
-    </x:r>
-    <x:r>
-      <x:rPr>
-        <x:u val="single"/>
-        <x:vertAlign val="baseline"/>
-        <x:sz val="11"/>
-        <x:color rgb="FFFF0000"/>
-        <x:rFont val="Calibri"/>
-        <x:family val="2"/>
-      </x:rPr>
-      <x:t>o</x:t>
-    </x:r>
-    <x:r>
-      <x:rPr>
-        <x:b/>
-        <x:u val="single"/>
-        <x:vertAlign val="baseline"/>
-        <x:sz val="11"/>
-        <x:color rgb="FF0000FF"/>
-        <x:rFont val="Calibri"/>
-        <x:family val="2"/>
-      </x:rPr>
-      <x:t xml:space="preserve"> BIG </x:t>
-    </x:r>
-    <x:r>
-      <x:rPr>
-        <x:u val="single"/>
-        <x:vertAlign val="baseline"/>
-        <x:sz val="11"/>
-        <x:color rgb="FFFF0000"/>
-        <x:rFont val="Calibri"/>
-        <x:family val="2"/>
-      </x:rPr>
-      <x:t>W</x:t>
-    </x:r>
-    <x:r>
-      <x:rPr>
-        <x:vertAlign val="baseline"/>
-        <x:sz val="11"/>
-        <x:color rgb="FFFF0000"/>
-        <x:rFont val="Calibri"/>
-        <x:family val="2"/>
-      </x:rPr>
-      <x:t>orld</x:t>
-    </x:r>
+    <x:t>" BIG " is Bold.</x:t>
   </x:si>
   <x:si>
     <x:r>
@@ -568,10 +568,10 @@
     </x:row>
     <x:row r="3" spans="1:2">
       <x:c r="A3" s="0" t="s">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:2">

</xml_diff>